<commit_message>
Sync local changes incl. RHEL8/9 verdict-logic fixes to phase1-phase2
</commit_message>
<xml_diff>
--- a/docs/01-product/use-cases/MD_Usecases_Implementation_Assessment.xlsx
+++ b/docs/01-product/use-cases/MD_Usecases_Implementation_Assessment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinay\Documents\ecs-enterprise-backup\docs\01-product\use-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8239503-C471-413F-BA6E-E9820B7D7001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50BB5323-46F1-401F-81D4-BAFE555D8304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1699,18 +1699,8 @@
   <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="36.15625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="60.89453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="55.15625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="81.3671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.62890625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="255.578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="101.20703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="255.578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="91.26171875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="126.9453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="26.3125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="80.26171875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="41.41796875" customWidth="1"/>
+    <col min="3" max="3" width="48.15625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.55000000000000004">

</xml_diff>